<commit_message>
Stabilize Wormsoft routing and extend cost guardrails
Refine Wormsoft throttle handling to avoid false provider outages, add credit-window pacing controls, and extend observability/tests for safer fallback behavior under load.
</commit_message>
<xml_diff>
--- a/docs/llm-cost-scenarios.xlsx
+++ b/docs/llm-cost-scenarios.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Routing" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Free risks" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Scale_2-3k" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="249">
   <si>
     <t xml:space="preserve">Frontier Intelligence — LLM cost assumptions</t>
   </si>
@@ -618,15 +619,173 @@
   </si>
   <si>
     <t xml:space="preserve">Окупается за 1 мес. Не «кредит на запросы», только разблокирует 1000 RPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бюджет токенов при росте 2000-3000 постов/день — GigaChat Lite/Pro/Max + EmbeddingsGigaR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сценарии объёма</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000/день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000/день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Постов в день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Постов в месяц</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Постов с картинками (30%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP synthesis вызовов / мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing signals probes / мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бюджет токенов на одну операцию (берём из shared/config.py + .env)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vision (на постах с картинкой)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Месячный объём токенов по задаче (M = миллионов)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000/день — Input M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000/день — Output M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000/день — Input M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000/день — Output M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Какому tier'у логично</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite (с fallback на Pro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EmbeddingsGigaR (отдельная модель, 2560d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pro (Lite не умеет vision)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pro (для качества синтеза)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИТОГО</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Распределение по моделям GigaChat (рекомендуемое: Lite + Pro для vision/mcp + Embed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена ₽/1M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2000/день — ₽/мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000/день — ₽/мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GigaChat-2 (Lite)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GigaChat-2-Pro (vision + mcp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИТОГО (рекомендуемый mix)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сравнение «всё на одной модели» (без рекомендуемого mix)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стратегия</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Текст M (in+out)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vision M (in+out)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embed M (in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₽/мес @ 2000/день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₽/мес @ 3000/день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Всё на GigaChat-2 (Lite) — vision НЕВОЗМОЖЕН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite-first (vision вынужденно на Pro 500₽/1M)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite 200, Pro 500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Всё на GigaChat-2-Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Всё на GigaChat-2-Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рекомендуемый mix (Lite + Pro vision/mcp + Embed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GigaChat-2 (Lite) НЕ имеет vision capabilities. Картинки можно обработать только Pro или Max — поэтому в строке «всё на Lite» vision = 0 (на практике придётся всё равно держать Pro для vision).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Embed — отдельная модель EmbeddingsGigaR (2560d), не учитывается в чат-моделях. Если использовать GigaEmbeddings-3B-2025-09 — цена ~50₽/1M такая же.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цены input/output у GigaChat одинаковые, поэтому в формулах сумма (input+output) × цена.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP synthesis и missing_signals масштабируются вместе с объёмом потока, но не строго пропорционально постам — здесь принято ×2 относительно baseline 500/день (50→100→150 для MCP, 20→40→60 для missing).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сравнение «pay-as-you-go GigaChat» vs «Wormsoft Simple subscription» (1500₽ держит ~72M кредитов): на 60-90M токенов чисто текста Wormsoft Simple перекрывает с большим запасом, GigaChat дороже минимум в ×30-50 на той же нагрузке.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При росте до 3000 постов/день рекомендация сменить FRONTIER_RUNTIME_MODE с balanced на gigachat-2-only НЕ имеет смысла — экономии не даст, выгоднее держать гибрид Wormsoft Simple + Pro для vision (см. лист Scenarios, S4).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Для real-time контроля бюджета: смотри Prometheus метрики gigachat_balance_remaining{type='pro'}, wormsoft_credits_remaining{plan='simple'}.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; ₽&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0&quot; ₽&quot;"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -763,7 +922,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -826,6 +985,26 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2799,4 +2978,842 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <f aca="false">B5*30</f>
+        <v>60000</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <f aca="false">C5*30</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <f aca="false">B6*0.3</f>
+        <v>18000</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <f aca="false">C6*0.3</f>
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <f aca="false">$B$6*B13/1000000</f>
+        <v>108</v>
+      </c>
+      <c r="C23" s="1" t="n">
+        <f aca="false">$B$6*C13/1000000</f>
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <f aca="false">$C$6*B13/1000000</f>
+        <v>162</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <f aca="false">$C$6*C13/1000000</f>
+        <v>27</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <f aca="false">$B$6*B14/1000000</f>
+        <v>72</v>
+      </c>
+      <c r="C24" s="1" t="n">
+        <f aca="false">$B$6*C14/1000000</f>
+        <v>12</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <f aca="false">$C$6*B14/1000000</f>
+        <v>108</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <f aca="false">$C$6*C14/1000000</f>
+        <v>18</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <f aca="false">$B$6*B15/1000000</f>
+        <v>72</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <f aca="false">$C$6*B15/1000000</f>
+        <v>108</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <f aca="false">$B$7*B16/1000000</f>
+        <v>46.8</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <f aca="false">$B$7*C16/1000000</f>
+        <v>7.2</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <f aca="false">$C$7*B16/1000000</f>
+        <v>70.2</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <f aca="false">$C$7*C16/1000000</f>
+        <v>10.8</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <f aca="false">$B$8*B17/1000000</f>
+        <v>12</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <f aca="false">$B$8*C17/1000000</f>
+        <v>4.5</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <f aca="false">$C$8*B17/1000000</f>
+        <v>18</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <f aca="false">$C$8*C17/1000000</f>
+        <v>6.75</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <f aca="false">$B$9*B18/1000000</f>
+        <v>6</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <f aca="false">$B$9*C18/1000000</f>
+        <v>1.2</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <f aca="false">$C$9*B18/1000000</f>
+        <v>9</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <f aca="false">$C$9*C18/1000000</f>
+        <v>1.8</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B29" s="8" t="n">
+        <f aca="false">SUM(B23:B28)</f>
+        <v>316.8</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <f aca="false">SUM(C23:C28)</f>
+        <v>42.9</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <f aca="false">SUM(D23:D28)</f>
+        <v>475.2</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <f aca="false">SUM(E23:E28)</f>
+        <v>64.35</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="C33" s="1" t="n">
+        <f aca="false">B23+B24+B28</f>
+        <v>186</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <f aca="false">C23+C24+C28</f>
+        <v>31.2</v>
+      </c>
+      <c r="E33" s="16" t="n">
+        <f aca="false">(C33+D33)*B33</f>
+        <v>43440</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <f aca="false">D23+D24+D28</f>
+        <v>279</v>
+      </c>
+      <c r="G33" s="16" t="n">
+        <f aca="false">E23+E24+E28</f>
+        <v>46.8</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <f aca="false">(F33+G33)*B33</f>
+        <v>65160</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="C34" s="1" t="n">
+        <f aca="false">B26+B27</f>
+        <v>58.8</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <f aca="false">C26+C27</f>
+        <v>11.7</v>
+      </c>
+      <c r="E34" s="16" t="n">
+        <f aca="false">(C34+D34)*B34</f>
+        <v>35250</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <f aca="false">D26+D27</f>
+        <v>88.2</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <f aca="false">E26+E27</f>
+        <v>17.55</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <f aca="false">(F34+G34)*B34</f>
+        <v>52875</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="C35" s="1" t="n">
+        <f aca="false">B25</f>
+        <v>72</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <f aca="false">C25</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="16" t="n">
+        <f aca="false">(C35+D35)*B35</f>
+        <v>3600</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <f aca="false">D25</f>
+        <v>108</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <f aca="false">E25</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="16" t="n">
+        <f aca="false">(F35+G35)*B35</f>
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="E36" s="18" t="n">
+        <f aca="false">SUM(E33:E35)</f>
+        <v>82290</v>
+      </c>
+      <c r="H36" s="18" t="n">
+        <f aca="false">SUM(H33:H35)</f>
+        <v>123435</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+    </row>
+    <row r="39" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="C40" s="1" t="n">
+        <f aca="false">(B23+C23+B24+C24+B27+C27+B28+C28)</f>
+        <v>233.7</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <f aca="false">B25</f>
+        <v>72</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <f aca="false">C40*B40+E40*50</f>
+        <v>50340</v>
+      </c>
+      <c r="G40" s="16" t="n">
+        <f aca="false">(D23+E23+D24+E24+D27+E27+D28+E28)*B40 + D25*50</f>
+        <v>75510</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C41" s="1" t="n">
+        <f aca="false">(B23+C23+B24+C24+B27+C27+B28+C28)</f>
+        <v>233.7</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <f aca="false">(B26+C26)</f>
+        <v>54</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <f aca="false">B25</f>
+        <v>72</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <f aca="false">C41*200 + D41*500 + E41*50</f>
+        <v>77340</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <f aca="false">(D23+E23+D24+E24+D27+E27+D28+E28)*200 + (D26+E26)*500 + D25*50</f>
+        <v>116010</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <f aca="false">(B23+C23+B24+C24+B27+C27+B28+C28)</f>
+        <v>233.7</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <f aca="false">(B26+C26)</f>
+        <v>54</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <f aca="false">B25</f>
+        <v>72</v>
+      </c>
+      <c r="F42" s="19" t="n">
+        <f aca="false">C42*B42+D42*B42+E42*50</f>
+        <v>147450</v>
+      </c>
+      <c r="G42" s="19" t="n">
+        <f aca="false">(D23+E23+D24+E24+D27+E27+D28+E28)*B42 + (D26+E26)*B42 + D25*50</f>
+        <v>221175</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C43" s="1" t="n">
+        <f aca="false">(B23+C23+B24+C24+B27+C27+B28+C28)</f>
+        <v>233.7</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <f aca="false">(B26+C26)</f>
+        <v>54</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <f aca="false">B25</f>
+        <v>72</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <f aca="false">C43*B43+D43*B43+E43*50</f>
+        <v>435150</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <f aca="false">(D23+E23+D24+E24+D27+E27+D28+E28)*B43 + (D26+E26)*B43 + D25*50</f>
+        <v>652725</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="F44" s="18" t="n">
+        <f aca="false">E36</f>
+        <v>82290</v>
+      </c>
+      <c r="G44" s="18" t="n">
+        <f aca="false">H36</f>
+        <v>123435</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20"/>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="20"/>
+      <c r="I45" s="20"/>
+    </row>
+    <row r="46" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+    </row>
+    <row r="47" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+    </row>
+    <row r="48" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="14"/>
+    </row>
+    <row r="49" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+    </row>
+    <row r="50" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="14"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="14"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="14"/>
+    </row>
+    <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+    </row>
+    <row r="52" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="s">
+        <v>248</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A51:I51"/>
+    <mergeCell ref="A52:I52"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>